<commit_message>
Implement PESV accident report demo functionality and update tests
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/attached_assets/DEMO-PRUEBA_muestra_informe_siniestros_PESV.xlsx
+++ b/attached_assets/DEMO-PRUEBA_muestra_informe_siniestros_PESV.xlsx
@@ -424,12 +424,12 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Empresa: DEMO-PRUEBA | MUESTRA FUNCIONAL NO OFICIAL · NIT: 900000000-0</v>
+        <v>Empresa: DEMO-PRUEBA · NIT: 900000000-0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Generado: 9/10/2026, 9:00:00 a. m.</v>
+        <v>Generado: 9/10/2026, 10:18:01 a. m. · Período consultado: 09/10/2026 al 09/10/2026</v>
       </c>
     </row>
     <row r="5">

</xml_diff>